<commit_message>
IMPLEMENTACION DE LOGICA DE PROCESAMIENTO DE LA EMPRESA ABSA
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/UBICACIONES GEOGRAFICAS POR DEPENDENCIA Y EMPRESA.xlsx
+++ b/Control de Facturas/Assets/Plantillas/UBICACIONES GEOGRAFICAS POR DEPENDENCIA Y EMPRESA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89329A4A-F518-442E-A8D0-A38736FFE13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684C034C-9936-4600-BF75-092A31E6B87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-60" windowWidth="20730" windowHeight="11040" xr2:uid="{9A68B20D-27EF-4CE0-A54E-40698DBEA5EB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9A68B20D-27EF-4CE0-A54E-40698DBEA5EB}"/>
   </bookViews>
   <sheets>
     <sheet name="UBICACIONES GEOGRAFICAS" sheetId="1" r:id="rId1"/>
@@ -871,7 +871,16 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1602,7 +1611,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>17</v>
       </c>
@@ -1616,7 +1625,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>18</v>
       </c>
@@ -2008,31 +2017,31 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="5" t="s">
+    <row r="59" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B59" s="5">
-        <v>0</v>
-      </c>
-      <c r="C59" s="5">
+      <c r="B59" s="6">
+        <v>30515637210</v>
+      </c>
+      <c r="C59" s="6">
         <v>770</v>
       </c>
-      <c r="D59" s="5">
+      <c r="D59" s="6">
         <v>54</v>
       </c>
     </row>
-    <row r="60" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="5" t="s">
+    <row r="60" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B60" s="5">
-        <v>0</v>
-      </c>
-      <c r="C60" s="5">
+      <c r="B60" s="6">
+        <v>30515637210</v>
+      </c>
+      <c r="C60" s="6">
         <v>956</v>
       </c>
-      <c r="D60" s="5">
+      <c r="D60" s="6">
         <v>22</v>
       </c>
     </row>
@@ -3142,31 +3151,31 @@
         <v>14</v>
       </c>
     </row>
-    <row r="140" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="5" t="s">
+    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B140" s="5">
-        <v>0</v>
-      </c>
-      <c r="C140" s="5">
+      <c r="B140" s="1">
+        <v>23138294404</v>
+      </c>
+      <c r="C140" s="1">
         <v>448</v>
       </c>
-      <c r="D140" s="5">
+      <c r="D140" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="141" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="5" t="s">
+    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B141" s="5">
-        <v>0</v>
-      </c>
-      <c r="C141" s="5">
+      <c r="B141" s="1">
+        <v>30637182907</v>
+      </c>
+      <c r="C141" s="1">
         <v>628</v>
       </c>
-      <c r="D141" s="5">
+      <c r="D141" s="1">
         <v>14</v>
       </c>
     </row>
@@ -3632,101 +3641,101 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="6" t="s">
+    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B175" s="6">
+      <c r="B175" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C175" s="6">
+      <c r="C175" s="1">
         <v>628</v>
       </c>
-      <c r="D175" s="6">
+      <c r="D175" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="176" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A176" s="6" t="s">
+    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B176" s="6">
+      <c r="B176" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C176" s="6">
+      <c r="C176" s="1">
         <v>969</v>
       </c>
-      <c r="D176" s="6">
+      <c r="D176" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="177" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A177" s="6" t="s">
+    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B177" s="6">
+      <c r="B177" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C177" s="6">
+      <c r="C177" s="1">
         <v>968</v>
       </c>
-      <c r="D177" s="6">
+      <c r="D177" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="178" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="6" t="s">
+    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B178" s="6">
+      <c r="B178" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C178" s="6">
+      <c r="C178" s="1">
         <v>987</v>
       </c>
-      <c r="D178" s="6">
+      <c r="D178" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="179" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A179" s="6" t="s">
+    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B179" s="6">
+      <c r="B179" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C179" s="6">
+      <c r="C179" s="1">
         <v>937</v>
       </c>
-      <c r="D179" s="6">
+      <c r="D179" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="180" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A180" s="6" t="s">
+    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B180" s="6">
+      <c r="B180" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C180" s="6">
+      <c r="C180" s="1">
         <v>1392</v>
       </c>
-      <c r="D180" s="6">
+      <c r="D180" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="181" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="6" t="s">
+    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B181" s="6">
+      <c r="B181" s="1">
         <v>30999027489</v>
       </c>
-      <c r="C181" s="6">
+      <c r="C181" s="1">
         <v>785</v>
       </c>
-      <c r="D181" s="6">
+      <c r="D181" s="1">
         <v>14</v>
       </c>
     </row>
@@ -3786,59 +3795,59 @@
         <v>6</v>
       </c>
     </row>
-    <row r="186" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="5" t="s">
+    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B186" s="5">
-        <v>0</v>
-      </c>
-      <c r="C186" s="5">
+      <c r="B186" s="1">
+        <v>30545788167</v>
+      </c>
+      <c r="C186" s="1">
         <v>949</v>
       </c>
-      <c r="D186" s="5">
+      <c r="D186" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="187" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A187" s="5" t="s">
+    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B187" s="5">
-        <v>0</v>
-      </c>
-      <c r="C187" s="5">
+      <c r="B187" s="1">
+        <v>30545788167</v>
+      </c>
+      <c r="C187" s="1">
         <v>951</v>
       </c>
-      <c r="D187" s="5">
+      <c r="D187" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="188" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A188" s="5" t="s">
+    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B188" s="5">
-        <v>0</v>
-      </c>
-      <c r="C188" s="5">
+      <c r="B188" s="1">
+        <v>30545788167</v>
+      </c>
+      <c r="C188" s="1">
         <v>796</v>
       </c>
-      <c r="D188" s="5">
+      <c r="D188" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="189" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A189" s="5" t="s">
+    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B189" s="5">
-        <v>0</v>
-      </c>
-      <c r="C189" s="5">
+      <c r="B189" s="1">
+        <v>30545788167</v>
+      </c>
+      <c r="C189" s="1">
         <v>952</v>
       </c>
-      <c r="D189" s="5">
+      <c r="D189" s="1">
         <v>82</v>
       </c>
     </row>
@@ -4531,9 +4540,7 @@
   </sheetData>
   <autoFilter ref="A1:D238" xr:uid="{CE4628DD-973B-45F7-8219-B8D49EAEB95B}">
     <filterColumn colId="1">
-      <filters>
-        <filter val="null"/>
-      </filters>
+      <colorFilter dxfId="0"/>
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>